<commit_message>
feat: chatbot + Dash no streamlit
</commit_message>
<xml_diff>
--- a/data_transform/quantidade_processos.xlsx
+++ b/data_transform/quantidade_processos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,17 +417,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nucleo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
@@ -448,37 +436,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5ª CC</t>
+          <t>1ª CC</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>703</v>
+        <v>713</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1ª CC</t>
+          <t>5ª CC</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>476</v>
+        <v>692</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -487,13 +475,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>466</v>
+        <v>487</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -502,13 +490,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>438</v>
+        <v>454</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -517,133 +505,133 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>347</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6ª CCJ</t>
+          <t>2ª CCJ</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>255</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7ª CC</t>
+          <t>1ª CCJ</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>251</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>5ª CCJ</t>
+          <t>7ª CC</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>239</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1ª CCJ</t>
+          <t>6ª CCJ</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2ª CCJ</t>
+          <t>4ª CCJ</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4ª CCJ</t>
+          <t>5ª CCJ</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>226</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3ª CCJ</t>
+          <t>2ª CC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>198</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2ª CC</t>
+          <t>3ª CCJ</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -652,7 +640,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
resolvendo lentidao do Bi
</commit_message>
<xml_diff>
--- a/data_transform/quantidade_processos.xlsx
+++ b/data_transform/quantidade_processos.xlsx
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -445,13 +445,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1485</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -460,13 +460,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>810</v>
+        <v>799</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -475,13 +475,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>714</v>
+        <v>703</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -496,7 +496,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -505,13 +505,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>575</v>
+        <v>578</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -520,13 +520,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -535,13 +535,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -550,13 +550,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -565,43 +565,43 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4ª CCJ</t>
+          <t>7ª CC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7ª CC</t>
+          <t>4ª CCJ</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -610,13 +610,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -640,13 +640,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>120</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>23/08/2026</t>
+          <t>24/08/2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">

</xml_diff>